<commit_message>
feat: integrate health department primary cohort (N=7) and restructure findings for CEO review meeting
</commit_message>
<xml_diff>
--- a/AIGGPA_Fieldwork_Review/04_AIGGPA_Master_Descriptive_Statistics.xlsx
+++ b/AIGGPA_Fieldwork_Review/04_AIGGPA_Master_Descriptive_Statistics.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -548,10 +548,10 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.09</v>
+        <v>3.11</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>3</v>
@@ -566,16 +566,16 @@
         <v>5</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>3.09</v>
+        <v>4.15</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>0</v>
+        <v>3.77</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>0</v>
+        <v>3.31</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -585,16 +585,16 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>3.21</v>
+        <v>3.19</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>1</v>
@@ -603,16 +603,16 @@
         <v>5</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>3.21</v>
+        <v>4.54</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0</v>
+        <v>3.8</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>0</v>
+        <v>3.35</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>0</v>
+        <v>2.21</v>
       </c>
     </row>
     <row r="4">
@@ -622,16 +622,16 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>3.11</v>
+        <v>3.09</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>3</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.98</v>
+        <v>1.02</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>1</v>
@@ -640,16 +640,16 @@
         <v>5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>3.11</v>
+        <v>4.46</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0</v>
+        <v>4.03</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>0</v>
+        <v>2.98</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>0</v>
+        <v>2.21</v>
       </c>
     </row>
     <row r="5">
@@ -659,16 +659,16 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>2.94</v>
+        <v>2.92</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>1.08</v>
+        <v>1.11</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>1</v>
@@ -677,16 +677,16 @@
         <v>5</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>2.94</v>
+        <v>4.54</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>0</v>
+        <v>3.53</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0</v>
+        <v>3.07</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>0</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="6">
@@ -696,16 +696,16 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>3.04</v>
+        <v>3.06</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>3</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>1.34</v>
+        <v>1.33</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>1</v>
@@ -714,16 +714,16 @@
         <v>5</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>3.04</v>
+        <v>1.08</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>0</v>
+        <v>1.87</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>0</v>
+        <v>3.02</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>0</v>
+        <v>4.52</v>
       </c>
     </row>
     <row r="7">
@@ -733,10 +733,10 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>3.02</v>
+        <v>3</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>3</v>
@@ -751,16 +751,16 @@
         <v>5</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>3.02</v>
+        <v>4.85</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>0</v>
+        <v>4.13</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0</v>
+        <v>3.09</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>0</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="8">
@@ -770,16 +770,16 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2.87</v>
+        <v>2.9</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>3</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>1.28</v>
+        <v>1.25</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>1</v>
@@ -788,16 +788,16 @@
         <v>5</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>2.87</v>
+        <v>4.54</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>0</v>
+        <v>2.93</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>0</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="9">
@@ -807,16 +807,16 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>2.71</v>
+        <v>2.72</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>1.17</v>
+        <v>1.14</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>1</v>
@@ -825,16 +825,16 @@
         <v>5</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>2.71</v>
+        <v>4.31</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>0</v>
+        <v>3.53</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0</v>
+        <v>2.84</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>0</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="10">
@@ -844,16 +844,16 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.21</v>
+        <v>3.12</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>3</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>1.12</v>
+        <v>1.11</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>1</v>
@@ -862,16 +862,16 @@
         <v>5</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>3.21</v>
+        <v>4.46</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0</v>
+        <v>3.77</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>0</v>
+        <v>2.17</v>
       </c>
     </row>
     <row r="11">
@@ -881,34 +881,34 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C11" s="3" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="J11" s="3" t="n">
         <v>2.64</v>
       </c>
-      <c r="D11" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E11" s="3" t="n">
-        <v>1.19</v>
-      </c>
-      <c r="F11" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="H11" s="3" t="n">
-        <v>2.64</v>
-      </c>
-      <c r="I11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="K11" s="3" t="n">
-        <v>0</v>
+        <v>1.55</v>
       </c>
     </row>
     <row r="12">
@@ -918,16 +918,16 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>2.93</v>
+        <v>2.9</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>3</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>1.22</v>
+        <v>1.21</v>
       </c>
       <c r="F12" s="2" t="n">
         <v>1</v>
@@ -936,16 +936,16 @@
         <v>5</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>2.93</v>
+        <v>4.69</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>0</v>
+        <v>2.95</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>0</v>
+        <v>1.95</v>
       </c>
     </row>
     <row r="13">
@@ -955,10 +955,10 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>2.79</v>
+        <v>2.78</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>3</v>
@@ -973,16 +973,16 @@
         <v>5</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>2.79</v>
+        <v>4.38</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>0</v>
+        <v>3.67</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0</v>
+        <v>2.75</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>0</v>
+        <v>1.74</v>
       </c>
     </row>
     <row r="14">
@@ -992,16 +992,16 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>1.96</v>
+        <v>2</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>1.24</v>
+        <v>1.22</v>
       </c>
       <c r="F14" s="2" t="n">
         <v>1</v>
@@ -1010,16 +1010,16 @@
         <v>5</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>1.96</v>
+        <v>3</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0</v>
+        <v>2.83</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>0</v>
+        <v>1.82</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>0</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="15">
@@ -1029,16 +1029,16 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1.9</v>
+        <v>1.95</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>1.23</v>
+        <v>1.22</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>1</v>
@@ -1047,16 +1047,16 @@
         <v>5</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>1.9</v>
+        <v>3.54</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>0</v>
+        <v>2.73</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0</v>
+        <v>1.64</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>0</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="16">
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="C16" s="2" t="n">
         <v>2.76</v>
@@ -1075,7 +1075,7 @@
         <v>3</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>1.19</v>
+        <v>1.16</v>
       </c>
       <c r="F16" s="2" t="n">
         <v>1</v>
@@ -1084,16 +1084,16 @@
         <v>5</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>2.76</v>
+        <v>4.23</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>0</v>
+        <v>3.3</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>0</v>
+        <v>2.84</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>0</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="17">
@@ -1103,16 +1103,16 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>2.77</v>
+        <v>2.79</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>1.34</v>
+        <v>1.3</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>1</v>
@@ -1121,16 +1121,16 @@
         <v>5</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>2.77</v>
+        <v>4.62</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>0</v>
+        <v>3.83</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="18">
@@ -1140,16 +1140,16 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>2.53</v>
+        <v>2.57</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>3</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>1.18</v>
+        <v>1.16</v>
       </c>
       <c r="F18" s="2" t="n">
         <v>1</v>
@@ -1158,16 +1158,16 @@
         <v>5</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>2.53</v>
+        <v>3.92</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0</v>
+        <v>3.6</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>0</v>
+        <v>2.47</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="19">
@@ -1177,10 +1177,10 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>2.94</v>
+        <v>3.01</v>
       </c>
       <c r="D19" s="3" t="n">
         <v>3</v>
@@ -1195,16 +1195,16 @@
         <v>5</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>2.94</v>
+        <v>4.08</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>0</v>
+        <v>3.6</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>0</v>
+        <v>2.98</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>0</v>
+        <v>2.05</v>
       </c>
     </row>
     <row r="20">
@@ -1214,16 +1214,16 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>2.8</v>
+        <v>2.96</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>3</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>1.15</v>
+        <v>1.06</v>
       </c>
       <c r="F20" s="2" t="n">
         <v>1</v>
@@ -1232,16 +1232,16 @@
         <v>5</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>2.8</v>
+        <v>5</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>0</v>
+        <v>2.75</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="21">
@@ -1251,16 +1251,16 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>2.7</v>
+        <v>2.81</v>
       </c>
       <c r="D21" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.98</v>
+        <v>0.88</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>1</v>
@@ -1269,16 +1269,16 @@
         <v>4</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>0</v>
+        <v>2.88</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="22">
@@ -1288,16 +1288,16 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>3.25</v>
+        <v>3.3</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>3</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>1.12</v>
+        <v>0.99</v>
       </c>
       <c r="F22" s="2" t="n">
         <v>1</v>
@@ -1306,16 +1306,16 @@
         <v>5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>3.25</v>
+        <v>5</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>0</v>
+        <v>3.6</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>0</v>
+        <v>3.38</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -1325,16 +1325,16 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="C23" s="3" t="n">
-        <v>2.45</v>
+        <v>2.63</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>1.1</v>
+        <v>1.04</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>1</v>
@@ -1343,16 +1343,16 @@
         <v>4</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>2.45</v>
+        <v>4</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>0</v>
+        <v>2.75</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -1380,16 +1380,16 @@
         <v>5</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>3.83</v>
+        <v>2.33</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>0</v>
+        <v>3.3</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>0</v>
+        <v>3.82</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>0</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="25">
@@ -1417,16 +1417,16 @@
         <v>5</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>2.83</v>
+        <v>1.33</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>0</v>
+        <v>3.12</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>0</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="26">
@@ -1454,16 +1454,16 @@
         <v>5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>2.3</v>
+        <v>3.67</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>0</v>
+        <v>2.06</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="27">
@@ -1491,16 +1491,16 @@
         <v>5</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>3.21</v>
+        <v>4.75</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>0</v>
+        <v>4.07</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>0</v>
+        <v>3.43</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>0</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="28">
@@ -1528,15 +1528,89 @@
         <v>5</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>2.79</v>
+        <v>1.5</v>
       </c>
       <c r="I28" s="2" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J28" s="2" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="K28" s="2" t="n">
+        <v>4.22</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Q78_ANMOL_ABHA</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H29" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J28" s="2" t="n">
+      <c r="I29" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="K28" s="2" t="n">
+      <c r="J29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Q79_IHIP_workload</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1552,7 +1626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1591,10 +1665,10 @@
         </is>
       </c>
       <c r="B3" s="6" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>30</v>
+        <v>29.9</v>
       </c>
     </row>
     <row r="4">
@@ -1607,7 +1681,7 @@
         <v>42</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>30</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="5">
@@ -1620,7 +1694,7 @@
         <v>31</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>22.1</v>
+        <v>20.1</v>
       </c>
     </row>
     <row r="6">
@@ -1630,10 +1704,10 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>13.6</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="7">
@@ -1646,432 +1720,447 @@
         <v>6</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>4.3</v>
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>2.6</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Yes, strongly agree</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Yes, somewhat</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Q19_Mandate</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n">
-        <v>78</v>
-      </c>
-      <c r="C11" s="6" t="n">
-        <v>55.7</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="B14" s="6" t="n">
+        <v>87</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>56.5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Don't Know</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B15" s="6" t="n">
         <v>39</v>
       </c>
-      <c r="C12" s="6" t="n">
-        <v>27.9</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="C15" s="6" t="n">
+        <v>25.3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="C13" s="6" t="n">
-        <v>16.4</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Q20_Devices</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
+      <c r="B16" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>17.5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>desktop, phone</t>
+          <t>Don't know</t>
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>43</v>
+        <v>1</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>30.7</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>phone only</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="n">
-        <v>27</v>
-      </c>
-      <c r="C18" s="6" t="n">
-        <v>19.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>phone, shared desktop</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="C19" s="6" t="n">
-        <v>16.4</v>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Q20_Devices</t>
+        </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>shared phone</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="C20" s="6" t="n">
-        <v>10.7</v>
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>desktop, laptop, phone</t>
+          <t>desktop, phone</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="C21" s="6" t="n">
-        <v>10</v>
+        <v>30.5</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>laptop, phone</t>
+          <t>phone only</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C22" s="6" t="n">
-        <v>6.4</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>desktop, laptop, tablet, phone</t>
+          <t>phone, shared desktop</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="C23" s="6" t="n">
-        <v>3.6</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>laptop, tablet, phone</t>
+          <t>desktop, laptop, phone</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>2.9</v>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>shared phone</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>9.699999999999999</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Q23_Outages</t>
-        </is>
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>laptop, phone</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>5.8</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>desktop, laptop, tablet, phone</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>3.2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Sometimes</t>
+          <t>phone</t>
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="C28" s="6" t="n">
-        <v>35.7</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Often</t>
+          <t>laptop, tablet, phone</t>
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="C29" s="6" t="n">
-        <v>24.3</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Rarely</t>
+          <t>phone, laptop</t>
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="C30" s="6" t="n">
-        <v>23.6</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Very often</t>
+          <t>desktop, phone, laptop</t>
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="C31" s="6" t="n">
-        <v>9.300000000000001</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>Never</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="C32" s="6" t="n">
-        <v>7.1</v>
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Q23_Outages</t>
+        </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>Q24_Helpdesk</t>
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Sometimes</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>34.4</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Often</t>
         </is>
       </c>
       <c r="B36" s="6" t="n">
-        <v>75</v>
+        <v>38</v>
       </c>
       <c r="C36" s="6" t="n">
-        <v>53.6</v>
+        <v>24.7</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Rarely</t>
         </is>
       </c>
       <c r="B37" s="6" t="n">
-        <v>65</v>
+        <v>33</v>
       </c>
       <c r="C37" s="6" t="n">
-        <v>46.4</v>
+        <v>21.4</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Very often</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="C38" s="6" t="n">
+        <v>8.4</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>Q27_PctDigital</t>
-        </is>
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Never</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C39" s="6" t="n">
+        <v>6.5</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C40" s="6" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Q24_Helpdesk</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="B40" s="5" t="inlineStr">
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C40" s="5" t="inlineStr">
+      <c r="C43" s="5" t="inlineStr">
         <is>
           <t>%</t>
         </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>61-80%</t>
-        </is>
-      </c>
-      <c r="B41" s="6" t="n">
-        <v>36</v>
-      </c>
-      <c r="C41" s="6" t="n">
-        <v>25.7</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>0-20%</t>
-        </is>
-      </c>
-      <c r="B42" s="6" t="n">
-        <v>34</v>
-      </c>
-      <c r="C42" s="6" t="n">
-        <v>24.3</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>41-60%</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="n">
-        <v>31</v>
-      </c>
-      <c r="C43" s="6" t="n">
-        <v>22.1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>21-40%</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="B44" s="6" t="n">
-        <v>27</v>
+        <v>84</v>
       </c>
       <c r="C44" s="6" t="n">
-        <v>19.3</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>81-100%</t>
+          <t>No</t>
         </is>
       </c>
       <c r="B45" s="6" t="n">
-        <v>12</v>
+        <v>70</v>
       </c>
       <c r="C45" s="6" t="n">
-        <v>8.6</v>
+        <v>45.5</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>Q36_NonGovtApps</t>
+          <t>Q27_PctDigital</t>
         </is>
       </c>
     </row>
@@ -2095,222 +2184,222 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>0-20%</t>
         </is>
       </c>
       <c r="B49" s="6" t="n">
-        <v>106</v>
+        <v>39</v>
       </c>
       <c r="C49" s="6" t="n">
-        <v>75.7</v>
+        <v>25.3</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
+          <t>61-80%</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="C50" s="6" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>41-60%</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="C51" s="6" t="n">
+        <v>20.8</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>21-40%</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="C52" s="6" t="n">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>81-100%</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="C53" s="6" t="n">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Q36_NonGovtApps</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="n">
+        <v>116</v>
+      </c>
+      <c r="C57" s="6" t="n">
+        <v>75.3</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B50" s="6" t="n">
-        <v>34</v>
-      </c>
-      <c r="C50" s="6" t="n">
-        <v>24.3</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
+      <c r="B58" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="C58" s="6" t="n">
+        <v>24.7</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>Q44_Training</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="B53" s="5" t="inlineStr">
+      <c r="B61" s="5" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C53" s="5" t="inlineStr">
+      <c r="C61" s="5" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="6" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B54" s="6" t="n">
-        <v>79</v>
-      </c>
-      <c r="C54" s="6" t="n">
-        <v>56.4</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="6" t="inlineStr">
+      <c r="B62" s="6" t="n">
+        <v>84</v>
+      </c>
+      <c r="C62" s="6" t="n">
+        <v>54.5</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="B55" s="6" t="n">
-        <v>61</v>
-      </c>
-      <c r="C55" s="6" t="n">
-        <v>43.6</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
+      <c r="B63" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="C63" s="6" t="n">
+        <v>45.5</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
         <is>
           <t>Q50_BeyondSkill</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="B58" s="5" t="inlineStr">
+      <c r="B66" s="5" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C58" s="5" t="inlineStr">
+      <c r="C66" s="5" t="inlineStr">
         <is>
           <t>%</t>
         </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="B59" s="6" t="n">
-        <v>72</v>
-      </c>
-      <c r="C59" s="6" t="n">
-        <v>51.4</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B60" s="6" t="n">
-        <v>68</v>
-      </c>
-      <c r="C60" s="6" t="n">
-        <v>48.6</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="4" t="inlineStr">
-        <is>
-          <t>Q61_PaperPct</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="B63" s="5" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="6" t="inlineStr">
-        <is>
-          <t>41-60%</t>
-        </is>
-      </c>
-      <c r="B64" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="C64" s="6" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="6" t="inlineStr">
-        <is>
-          <t>81-100%</t>
-        </is>
-      </c>
-      <c r="B65" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="C65" s="6" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="6" t="inlineStr">
-        <is>
-          <t>61-80%</t>
-        </is>
-      </c>
-      <c r="B66" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="C66" s="6" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>21-40%</t>
+          <t>No</t>
         </is>
       </c>
       <c r="B67" s="6" t="n">
-        <v>2</v>
+        <v>81</v>
       </c>
       <c r="C67" s="6" t="n">
-        <v>10</v>
+        <v>52.6</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>0-20%</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="B68" s="6" t="n">
-        <v>1</v>
+        <v>73</v>
       </c>
       <c r="C68" s="6" t="n">
-        <v>5</v>
+        <v>47.4</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>Q69_DataEntryTime</t>
+          <t>Q61_PaperPct</t>
         </is>
       </c>
     </row>
@@ -2334,72 +2423,72 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>1-2 hours</t>
+          <t>41-60%</t>
         </is>
       </c>
       <c r="B72" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C72" s="6" t="n">
-        <v>32.5</v>
+        <v>40.7</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>30-60 min</t>
+          <t>81-100%</t>
         </is>
       </c>
       <c r="B73" s="6" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C73" s="6" t="n">
-        <v>22.5</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>&gt;2 hours</t>
+          <t>21-40%</t>
         </is>
       </c>
       <c r="B74" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C74" s="6" t="n">
-        <v>20</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>&lt;15 min</t>
+          <t>61-80%</t>
         </is>
       </c>
       <c r="B75" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C75" s="6" t="n">
-        <v>12.5</v>
+        <v>14.8</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>15-30 min</t>
+          <t>0-20%</t>
         </is>
       </c>
       <c r="B76" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C76" s="6" t="n">
-        <v>12.5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>Q71_PortalDown</t>
+          <t>Q69_DataEntryTime</t>
         </is>
       </c>
     </row>
@@ -2423,155 +2512,307 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>Switch to manual register and upload later</t>
+          <t>1-2 hours</t>
         </is>
       </c>
       <c r="B80" s="6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C80" s="6" t="n">
-        <v>25</v>
+        <v>32.5</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>Use mobile data and try again</t>
+          <t>30-60 min</t>
         </is>
       </c>
       <c r="B81" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C81" s="6" t="n">
-        <v>25</v>
+        <v>22.5</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>Call block office for help</t>
+          <t>&gt;2 hours</t>
         </is>
       </c>
       <c r="B82" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C82" s="6" t="n">
-        <v>22.5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>Wait and retry after some time</t>
+          <t>&lt;15 min</t>
         </is>
       </c>
       <c r="B83" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C83" s="6" t="n">
-        <v>15</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>Skip the task for the day</t>
+          <t>15-30 min</t>
         </is>
       </c>
       <c r="B84" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C84" s="6" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>Q71_PortalDown</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t>Switch to manual register and upload later</t>
+        </is>
+      </c>
+      <c r="B88" s="6" t="n">
         <v>10</v>
       </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="6" t="inlineStr">
-        <is>
-          <t>Contact NIC helpdesk</t>
-        </is>
-      </c>
-      <c r="B85" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C85" s="6" t="n">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="4" t="inlineStr">
-        <is>
-          <t>Q75_GPSDevice</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="5" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="B88" s="5" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="C88" s="5" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
+      <c r="C88" s="6" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>Not available</t>
+          <t>Use mobile data and try again</t>
         </is>
       </c>
       <c r="B89" s="6" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C89" s="6" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>Personal device</t>
+          <t>Call block office for help</t>
         </is>
       </c>
       <c r="B90" s="6" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="C90" s="6" t="n">
-        <v>37.5</v>
+        <v>22.5</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>Dept-issued device</t>
+          <t>Wait and retry after some time</t>
         </is>
       </c>
       <c r="B91" s="6" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C91" s="6" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
+          <t>Skip the task for the day</t>
+        </is>
+      </c>
+      <c r="B92" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C92" s="6" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="inlineStr">
+        <is>
+          <t>Contact NIC helpdesk</t>
+        </is>
+      </c>
+      <c r="B93" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C93" s="6" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t>Q75_GPSDevice</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="6" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="B97" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="C97" s="6" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="inlineStr">
+        <is>
+          <t>Personal device</t>
+        </is>
+      </c>
+      <c r="B98" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="C98" s="6" t="n">
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="6" t="inlineStr">
+        <is>
+          <t>Dept-issued device</t>
+        </is>
+      </c>
+      <c r="B99" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="C99" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="6" t="inlineStr">
+        <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="B92" s="6" t="n">
+      <c r="B100" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="C92" s="6" t="n">
+      <c r="C100" s="6" t="n">
         <v>2.5</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="inlineStr">
+        <is>
+          <t>Q77_HealthTools</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="6" t="inlineStr">
+        <is>
+          <t>ANMOL MP</t>
+        </is>
+      </c>
+      <c r="B104" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C104" s="6" t="n">
+        <v>71.40000000000001</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
+          <t>ANMOL MP, eVIN</t>
+        </is>
+      </c>
+      <c r="B105" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C105" s="6" t="n">
+        <v>14.3</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="6" t="inlineStr">
+        <is>
+          <t>ANMOL MP, eVIN, HMIS</t>
+        </is>
+      </c>
+      <c r="B106" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C106" s="6" t="n">
+        <v>14.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>